<commit_message>
fix: stabilize workbook E2E packaging
</commit_message>
<xml_diff>
--- a/workbooks/source/BHA_Vibration_Bending_and_Drill_Ahead_Tendency_SI.xlsx
+++ b/workbooks/source/BHA_Vibration_Bending_and_Drill_Ahead_Tendency_SI.xlsx
@@ -726,152 +726,6 @@
         <c:axId val="148650112"/>
         <c:axId val="148672768"/>
       </c:radarChart>
-      <c:scatterChart>
-        <c:scatterStyle val="lineMarker"/>
-        <c:ser>
-          <c:idx val="0"/>
-          <c:order val="0"/>
-          <c:tx>
-            <c:v>WOB 1</c:v>
-          </c:tx>
-          <c:spPr>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-              <a:solidFill>
-                <a:srgbClr val="0F766E">
-                  <a:alpha val="65000"/>
-                </a:srgbClr>
-              </a:solidFill>
-            </a:ln>
-          </c:spPr>
-          <c:xVal>
-            <c:numRef>
-              <c:f>='Polar Plot'!$B$6:$B$18</c:f>
-              <c:numCache>
-                <c:formatCode>General</c:formatCode>
-                <c:ptCount val="0"/>
-              </c:numCache>
-            </c:numRef>
-          </c:xVal>
-          <c:yVal>
-            <c:numRef>
-              <c:f>='Polar Plot'!$C$6:$C$18</c:f>
-              <c:numCache>
-                <c:formatCode>#,##0.00;[Red]-#,##0.00</c:formatCode>
-                <c:ptCount val="0"/>
-              </c:numCache>
-            </c:numRef>
-          </c:yVal>
-        </c:ser>
-        <c:ser>
-          <c:idx val="1"/>
-          <c:order val="1"/>
-          <c:tx>
-            <c:v>WOB 2</c:v>
-          </c:tx>
-          <c:spPr>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-              <a:solidFill>
-                <a:srgbClr val="D97706">
-                  <a:alpha val="65000"/>
-                </a:srgbClr>
-              </a:solidFill>
-            </a:ln>
-          </c:spPr>
-          <c:xVal>
-            <c:numRef>
-              <c:f>='Polar Plot'!$D$6:$D$18</c:f>
-              <c:numCache>
-                <c:formatCode>General</c:formatCode>
-                <c:ptCount val="0"/>
-              </c:numCache>
-            </c:numRef>
-          </c:xVal>
-          <c:yVal>
-            <c:numRef>
-              <c:f>='Polar Plot'!$E$6:$E$18</c:f>
-              <c:numCache>
-                <c:formatCode>#,##0.00;[Red]-#,##0.00</c:formatCode>
-                <c:ptCount val="0"/>
-              </c:numCache>
-            </c:numRef>
-          </c:yVal>
-        </c:ser>
-        <c:axId val="48650112"/>
-        <c:axId val="48672768"/>
-      </c:scatterChart>
-      <c:valAx>
-        <c:axId val="48672768"/>
-        <c:scaling>
-          <c:orientation val="minMax"/>
-        </c:scaling>
-        <c:delete val="0"/>
-        <c:axPos val="l"/>
-        <c:majorGridlines>
-          <c:spPr>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9525">
-              <a:solidFill>
-                <a:srgbClr val="CCCCCC"/>
-              </a:solidFill>
-              <a:prstDash val="dash"/>
-            </a:ln>
-          </c:spPr>
-        </c:majorGridlines>
-        <c:title>
-          <c:tx>
-            <c:rich>
-              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-              <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-                <a:r>
-                  <a:t>North component</a:t>
-                </a:r>
-              </a:p>
-            </c:rich>
-          </c:tx>
-          <c:overlay val="0"/>
-        </c:title>
-        <c:numFmt formatCode="#,##0.00;[Red]-#,##0.00" sourceLinked="0"/>
-        <c:majorTickMark val="none"/>
-        <c:minorTickMark val="none"/>
-        <c:crossAx val="48650112"/>
-      </c:valAx>
-      <c:valAx>
-        <c:axId val="48650112"/>
-        <c:scaling>
-          <c:orientation val="minMax"/>
-        </c:scaling>
-        <c:delete val="0"/>
-        <c:axPos val="b"/>
-        <c:majorGridlines>
-          <c:spPr>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9525">
-              <a:solidFill>
-                <a:srgbClr val="CCCCCC"/>
-              </a:solidFill>
-              <a:prstDash val="dash"/>
-            </a:ln>
-          </c:spPr>
-        </c:majorGridlines>
-        <c:title>
-          <c:tx>
-            <c:rich>
-              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-              <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-                <a:r>
-                  <a:t>East component</a:t>
-                </a:r>
-              </a:p>
-            </c:rich>
-          </c:tx>
-          <c:overlay val="0"/>
-        </c:title>
-        <c:numFmt formatCode="#,##0.00;[Red]-#,##0.00" sourceLinked="0"/>
-        <c:majorTickMark val="none"/>
-        <c:minorTickMark val="none"/>
-        <c:tickLblPos val="nextTo"/>
-        <c:crossAx val="48672768"/>
-      </c:valAx>
       <c:catAx>
         <c:axId val="148650112"/>
         <c:scaling>
@@ -1478,6 +1332,190 @@
               <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:r>
                   <a:t>Frequency (Hz)</a:t>
+                </a:r>
+              </a:p>
+            </c:rich>
+          </c:tx>
+          <c:overlay val="0"/>
+        </c:title>
+        <c:numFmt formatCode="#,##0.00;[Red]-#,##0.00" sourceLinked="0"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:crossAx val="48672768"/>
+      </c:valAx>
+    </c:plotArea>
+    <c:legend>
+      <c:legendPos val="b"/>
+      <c:overlay val="0"/>
+    </c:legend>
+    <c:plotVisOnly val="1"/>
+  </c:chart>
+  <c:spPr>
+    <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9525">
+      <a:solidFill>
+        <a:srgbClr val="D9D9D9"/>
+      </a:solidFill>
+      <a:prstDash val="solid"/>
+    </a:ln>
+  </c:spPr>
+</c:chartSpace>
+</file>
+
+<file path=xl/drawings/charts/chart16.xml><?xml version="1.0" encoding="utf-8"?>
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart">
+  <c:lang val="en-US"/>
+  <c:roundedCorners val="0"/>
+  <c:chart>
+    <c:title>
+      <c:tx>
+        <c:rich>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:r>
+              <a:t>WOB/toolface polar response</a:t>
+            </a:r>
+          </a:p>
+        </c:rich>
+      </c:tx>
+      <c:overlay val="0"/>
+    </c:title>
+    <c:plotArea>
+      <c:scatterChart>
+        <c:scatterStyle val="lineMarker"/>
+        <c:ser>
+          <c:idx val="0"/>
+          <c:order val="0"/>
+          <c:tx>
+            <c:v>WOB 1</c:v>
+          </c:tx>
+          <c:spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:solidFill>
+                <a:srgbClr val="0F766E">
+                  <a:alpha val="65000"/>
+                </a:srgbClr>
+              </a:solidFill>
+            </a:ln>
+          </c:spPr>
+          <c:xVal>
+            <c:numRef>
+              <c:f>='Polar Plot'!$B$6:$B$18</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="0"/>
+              </c:numCache>
+            </c:numRef>
+          </c:xVal>
+          <c:yVal>
+            <c:numRef>
+              <c:f>='Polar Plot'!$C$6:$C$18</c:f>
+              <c:numCache>
+                <c:formatCode>#,##0.00;[Red]-#,##0.00</c:formatCode>
+                <c:ptCount val="0"/>
+              </c:numCache>
+            </c:numRef>
+          </c:yVal>
+        </c:ser>
+        <c:ser>
+          <c:idx val="1"/>
+          <c:order val="1"/>
+          <c:tx>
+            <c:v>WOB 2</c:v>
+          </c:tx>
+          <c:spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:solidFill>
+                <a:srgbClr val="D97706">
+                  <a:alpha val="65000"/>
+                </a:srgbClr>
+              </a:solidFill>
+            </a:ln>
+          </c:spPr>
+          <c:xVal>
+            <c:numRef>
+              <c:f>='Polar Plot'!$D$6:$D$18</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="0"/>
+              </c:numCache>
+            </c:numRef>
+          </c:xVal>
+          <c:yVal>
+            <c:numRef>
+              <c:f>='Polar Plot'!$E$6:$E$18</c:f>
+              <c:numCache>
+                <c:formatCode>#,##0.00;[Red]-#,##0.00</c:formatCode>
+                <c:ptCount val="0"/>
+              </c:numCache>
+            </c:numRef>
+          </c:yVal>
+        </c:ser>
+        <c:axId val="48650112"/>
+        <c:axId val="48672768"/>
+      </c:scatterChart>
+      <c:valAx>
+        <c:axId val="48672768"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="l"/>
+        <c:majorGridlines>
+          <c:spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9525">
+              <a:solidFill>
+                <a:srgbClr val="CCCCCC"/>
+              </a:solidFill>
+              <a:prstDash val="dash"/>
+            </a:ln>
+          </c:spPr>
+        </c:majorGridlines>
+        <c:title>
+          <c:tx>
+            <c:rich>
+              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:r>
+                  <a:t>North component</a:t>
+                </a:r>
+              </a:p>
+            </c:rich>
+          </c:tx>
+          <c:overlay val="0"/>
+        </c:title>
+        <c:numFmt formatCode="#,##0.00;[Red]-#,##0.00" sourceLinked="0"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:crossAx val="48650112"/>
+      </c:valAx>
+      <c:valAx>
+        <c:axId val="48650112"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="b"/>
+        <c:majorGridlines>
+          <c:spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9525">
+              <a:solidFill>
+                <a:srgbClr val="CCCCCC"/>
+              </a:solidFill>
+              <a:prstDash val="dash"/>
+            </a:ln>
+          </c:spPr>
+        </c:majorGridlines>
+        <c:title>
+          <c:tx>
+            <c:rich>
+              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:r>
+                  <a:t>East component</a:t>
                 </a:r>
               </a:p>
             </c:rich>
@@ -3581,6 +3619,36 @@
     </xdr:graphicFrame>
     <xdr:clientData/>
   </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>6</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>19</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>14</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>38</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:to>
+    <xdr:graphicFrame macro="">
+      <xdr:nvGraphicFramePr>
+        <xdr:cNvPr id="3" name="Chart 16"/>
+        <xdr:cNvGraphicFramePr/>
+      </xdr:nvGraphicFramePr>
+      <xdr:xfrm>
+        <a:off xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" x="0" y="0"/>
+        <a:ext xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" cx="0" cy="0"/>
+      </xdr:xfrm>
+      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="rId2"/>
+        </a:graphicData>
+      </a:graphic>
+    </xdr:graphicFrame>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
 </xdr:wsDr>
 </file>
 

</xml_diff>